<commit_message>
Update Customer Logic & UI
</commit_message>
<xml_diff>
--- a/data/customers.xlsx
+++ b/data/customers.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="140">
   <si>
     <t>Nama</t>
   </si>
@@ -430,6 +430,9 @@
   </si>
   <si>
     <t>82190876543</t>
+  </si>
+  <si>
+    <t>2023</t>
   </si>
 </sst>
 </file>
@@ -727,8 +730,8 @@
       <c r="F2" t="s" s="0">
         <v>11</v>
       </c>
-      <c r="G2" t="n" s="0">
-        <v>2023.0</v>
+      <c r="G2" t="s" s="0">
+        <v>139</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Update UI & Logic
</commit_message>
<xml_diff>
--- a/data/customers.xlsx
+++ b/data/customers.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="146">
   <si>
     <t>Nama</t>
   </si>
@@ -433,6 +433,24 @@
   </si>
   <si>
     <t>2023</t>
+  </si>
+  <si>
+    <t>Bayu Adi Nugroho</t>
+  </si>
+  <si>
+    <t>098</t>
+  </si>
+  <si>
+    <t>Mojokerto</t>
+  </si>
+  <si>
+    <t>B 4 Y U</t>
+  </si>
+  <si>
+    <t>Amfibi</t>
+  </si>
+  <si>
+    <t>2050</t>
   </si>
 </sst>
 </file>
@@ -685,7 +703,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
@@ -1401,6 +1419,29 @@
         <v>2024.0</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>140</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="C32" t="s" s="0">
+        <v>142</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>143</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F32" t="s" s="0">
+        <v>144</v>
+      </c>
+      <c r="G32" t="s" s="0">
+        <v>145</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>